<commit_message>
Update Readme und Projektplanung
</commit_message>
<xml_diff>
--- a/PMGT-ZZA.xlsx
+++ b/PMGT-ZZA.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erik\Documents\HAW\Bachelorprojekt\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erik\Documents\HAW\Bachelorprojekt\git\Zugzielanzeige\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6C055222-19A8-4404-BB65-F965F5911D6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6655FF96-0EA3-4079-9D6F-E190167C312C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Projektziele" sheetId="1" r:id="rId1"/>
@@ -23,8 +23,11 @@
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="1">Pflichtenheft!$B:$C</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -41,133 +44,197 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="108">
-  <si>
-    <t>Risiko</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="124">
+  <si>
+    <t>Projektziele</t>
+  </si>
+  <si>
+    <t>In diesem Dokument werden die Top-Level-Ziele des Projekts festgelegt. Es dient der Balancierung der verschiedenen Ziele und der Messung der Zielerreichung durch den Auftraggeber / das Management am Ende des Projekts.Typischerweise wird jeder Projektmanagement-Bereich (Qualität, Kosten, Zeit) mit mindestems einem Ziel belegt. Die Anzahl der Ziele und der Detaillierungsgrad sind eher gering (Management-Kompatibilität!), wo notwendig können Unterdokumente wie z.B. das Pflichtenheft referenziert werden.</t>
+  </si>
+  <si>
+    <t>Ziele</t>
   </si>
   <si>
     <t>Prio</t>
   </si>
   <si>
+    <t>quantitativ messbares Kriterium</t>
+  </si>
+  <si>
+    <t>Technik</t>
+  </si>
+  <si>
+    <t>Zeit</t>
+  </si>
+  <si>
+    <t>90% der im Zeitplan definierten Meilensteine inhaltlich und zeitlich erreicht.</t>
+  </si>
+  <si>
+    <t>Budget</t>
+  </si>
+  <si>
+    <t>…</t>
+  </si>
+  <si>
+    <t>Zusammenarbeit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sonstiges </t>
+  </si>
+  <si>
+    <t>Unterschriften der Team-Mitglieder</t>
+  </si>
+  <si>
+    <t>Unterschrift Auftraggeber</t>
+  </si>
+  <si>
+    <t>Pflichtenheft</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Das Pflichtenheft beschreibt alle technischen Eigenschaften des zu entwickelnden Produkts und ist daher typischerweise recht umfangreich. Um den Aufwand im Lernprojekt klein zu halten, soll ein reduziertes Dokument erstellt werden, an dem die Arbeit mit dem Pflichtenheft exemplarisch durchgeführt wird:
+1. Identifizieren Sie die drei wichtigsten Teilfunktionen Ihres ZZA. Definieren Sie für jede dieser drei Teilfunktionen die quantitativen Anforderungen, an denen die technische Zielerreichung gemessen wird. 
+Aus einem guten Pflichtenheft ergibt ich quasi automatisch ein Plan für den Labortest, in dem die Erreichung der technischen Ziele nachgewiesen wird. </t>
+  </si>
+  <si>
+    <t>Teilfunktion 1</t>
+  </si>
+  <si>
+    <t>Stromversorgung der ZZA</t>
+  </si>
+  <si>
+    <t>Kurzbeschreibung der Teilfunktion</t>
+  </si>
+  <si>
+    <t>Stromversorgung für alle Bauteile des ZZA. Soll sicher sein, dass niemand zu schaden kommt.</t>
+  </si>
+  <si>
     <t>Anforderung 1</t>
   </si>
   <si>
+    <t>Getrennte Erdung und Nulleiter</t>
+  </si>
+  <si>
+    <t>Anforderung 2</t>
+  </si>
+  <si>
+    <t>Spannungsversorgung an den Netzteilen</t>
+  </si>
+  <si>
     <t>Anforderung 3</t>
   </si>
   <si>
-    <t>Anforderung 2</t>
-  </si>
-  <si>
-    <t>Kurzbeschreibung der Teilfunktion</t>
-  </si>
-  <si>
-    <t>Teilfunktion 1</t>
+    <t>Durchgängigkeit des Schutzleiters</t>
+  </si>
+  <si>
+    <t>Teilfunktion 2</t>
+  </si>
+  <si>
+    <t>Ansteuerung der LED-Matrix</t>
+  </si>
+  <si>
+    <t>Kontrollierte Anzeigen durch LEDs, mit verschiedenen Farben und einer hohen Aktualisierungsrate um Flackern der LEDs zu verhindern.
+Higher level control über die LED-Matrix (Funktionen um z.B. Rechtecke/Linien/etc. anzuzeigen), ganze Reihen/Sektionen ansteuern</t>
+  </si>
+  <si>
+    <t>Kein erkennbares Flackern der LEDs</t>
+  </si>
+  <si>
+    <t>Einzelne LEDs ansteuerbar</t>
+  </si>
+  <si>
+    <t>Anforderung 4</t>
+  </si>
+  <si>
+    <t>Anforderung 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Higher level control über die LED-Matrix </t>
+  </si>
+  <si>
+    <t>Teilfunktion 3</t>
+  </si>
+  <si>
+    <t>Eingabegeräte (HID/PC)</t>
+  </si>
+  <si>
+    <t>Nutzen von Controller / Tastatur / Maus um elemente auf dem Display zu steuern. Datenübertragung vom PC aus (mit UART?)</t>
+  </si>
+  <si>
+    <t>Teilfunktion 4</t>
+  </si>
+  <si>
+    <t>Komplettes Spiel</t>
+  </si>
+  <si>
+    <t>Ein simples Spiel auf der ZZA laufen lassen, evtl. Zweispieler?</t>
+  </si>
+  <si>
+    <t>Projektorganisation</t>
+  </si>
+  <si>
+    <t>In der Projektorganisation sind die Rollen der Teammitglieder festgelegt. Sie klärt Verantwortlichkeiten und Schnittstellen (Hol- bzw. Bringschuld) und ggfs. auch Hierarchien. Eine gute Projektorganisation ist auf die Projektinhalte abgestimmt (z.B. Bildung von Teilprojektteams für zentrale Aspekte) und berücksichtigt die Stärken / Schwächen und Charaktereigenschaften der einzelnen Teammitglieder.</t>
+  </si>
+  <si>
+    <t>Zeitplan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Der Zeitplan zeigt, in welcher Abfolge die Arbeitspakete abgearbeitet werden. Dabei sind Vorgänger-Nachfolger-Beziehungen und Möglichkeiten zur Parallelisierung von Arbeitspaketen zu berücksichtigen. Meilensteine dienen zur Messung der inhaltlichen und zeitlichen Zielerreichung im Projektverlauf.
+sinnvolle Planungstiefe: Arbeitspakete ca. 1/2 Manntag, ca. ein Meilenstein pro Tag
+</t>
+  </si>
+  <si>
+    <t>Nr.</t>
+  </si>
+  <si>
+    <t>Arbeitspaket</t>
+  </si>
+  <si>
+    <t>verantwortlich</t>
+  </si>
+  <si>
+    <t>Mai</t>
+  </si>
+  <si>
+    <t>Juni</t>
+  </si>
+  <si>
+    <t>Juli</t>
+  </si>
+  <si>
+    <t>August</t>
+  </si>
+  <si>
+    <t>September</t>
   </si>
   <si>
     <t>Projektplanung</t>
   </si>
   <si>
+    <t>alle</t>
+  </si>
+  <si>
     <t>Projektplanung abgeschlossen</t>
   </si>
   <si>
     <t>Test und Optimierung</t>
   </si>
   <si>
-    <t>Abschlusspräsentation</t>
-  </si>
-  <si>
-    <t>Projektziele</t>
-  </si>
-  <si>
-    <t>…</t>
-  </si>
-  <si>
-    <t>Pflichtenheft</t>
-  </si>
-  <si>
-    <t>Unterschriften der Team-Mitglieder</t>
-  </si>
-  <si>
-    <t>Unterschrift Auftraggeber</t>
-  </si>
-  <si>
-    <t>Teilfunktion 2</t>
-  </si>
-  <si>
-    <t>Teilfunktion 3</t>
-  </si>
-  <si>
-    <t>Technik</t>
-  </si>
-  <si>
-    <t>Zeit</t>
-  </si>
-  <si>
-    <t>Budget</t>
-  </si>
-  <si>
-    <t>Zusammenarbeit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sonstiges </t>
+    <t>Das Projektbudget dient der Kostenprognose und -kontrolle. Zu Projektbeginn werden die geplanten Beschaffungen und die geschätzten Kosten eingetragen. Wenn Material gekauft wird, werden die geplanten Kosten in dieser Tabelle um die tatsächlich angefallenen Kosten ergänzt. Auf diese Weise können Kostenüberschreitungen frühzeitig erkannt und ggfs. Gegenmaßnahmen eingeleitet werden.</t>
+  </si>
+  <si>
+    <t>Position</t>
+  </si>
+  <si>
+    <t>Plankosten [€]</t>
+  </si>
+  <si>
+    <t>Zugzielanzeiger</t>
+  </si>
+  <si>
+    <t>Summe</t>
   </si>
   <si>
     <t>Risikoanalyse</t>
-  </si>
-  <si>
-    <t>Zeitplan</t>
-  </si>
-  <si>
-    <t>Nr.</t>
-  </si>
-  <si>
-    <t>Arbeitspaket</t>
-  </si>
-  <si>
-    <t>verantwortlich</t>
-  </si>
-  <si>
-    <t>Projektorganisation</t>
-  </si>
-  <si>
-    <t>Position</t>
-  </si>
-  <si>
-    <t>Summe</t>
-  </si>
-  <si>
-    <t>Plankosten [€]</t>
-  </si>
-  <si>
-    <t>Istkosten [€]</t>
-  </si>
-  <si>
-    <t>erledigt bis</t>
-  </si>
-  <si>
-    <t>Relevanz des Risikos</t>
-  </si>
-  <si>
-    <t>Gegenmaßnahme</t>
-  </si>
-  <si>
-    <t>Eintritts-
-wahrscheinlichkeit</t>
-  </si>
-  <si>
-    <t>Minderung des  Zielerreichungsgrades bei Risikoeintritt</t>
-  </si>
-  <si>
-    <t>Ziele</t>
-  </si>
-  <si>
-    <t>quantitativ messbares Kriterium</t>
-  </si>
-  <si>
-    <t>Bob der Baumeister</t>
-  </si>
-  <si>
-    <t>90% der im Zeitplan definierten Meilensteine inhaltlich und zeitlich erreicht.</t>
   </si>
   <si>
     <t>Die Risikoanalyse dient dem Management der Risiken. Wichtig ist:
@@ -176,93 +243,23 @@
 3. Die Festlegung und Umsetzung geeigneter Gegenmaßnahmen. Wirksame Gegenmaßnahmen reduzieren die Relevanz des Risikos auf einen akzeptablen Wert.</t>
   </si>
   <si>
-    <t xml:space="preserve">Der Zeitplan zeigt, in welcher Abfolge die Arbeitspakete abgearbeitet werden. Dabei sind Vorgänger-Nachfolger-Beziehungen und Möglichkeiten zur Parallelisierung von Arbeitspaketen zu berücksichtigen. Meilensteine dienen zur Messung der inhaltlichen und zeitlichen Zielerreichung im Projektverlauf.
-sinnvolle Planungstiefe: Arbeitspakete ca. 1/2 Manntag, ca. ein Meilenstein pro Tag
-</t>
-  </si>
-  <si>
-    <t>Das Projektbudget dient der Kostenprognose und -kontrolle. Zu Projektbeginn werden die geplanten Beschaffungen und die geschätzten Kosten eingetragen. Wenn Material gekauft wird, werden die geplanten Kosten in dieser Tabelle um die tatsächlich angefallenen Kosten ergänzt. Auf diese Weise können Kostenüberschreitungen frühzeitig erkannt und ggfs. Gegenmaßnahmen eingeleitet werden.</t>
-  </si>
-  <si>
-    <t>In der Projektorganisation sind die Rollen der Teammitglieder festgelegt. Sie klärt Verantwortlichkeiten und Schnittstellen (Hol- bzw. Bringschuld) und ggfs. auch Hierarchien. Eine gute Projektorganisation ist auf die Projektinhalte abgestimmt (z.B. Bildung von Teilprojektteams für zentrale Aspekte) und berücksichtigt die Stärken / Schwächen und Charaktereigenschaften der einzelnen Teammitglieder.</t>
-  </si>
-  <si>
-    <t>In diesem Dokument werden die Top-Level-Ziele des Projekts festgelegt. Es dient der Balancierung der verschiedenen Ziele und der Messung der Zielerreichung durch den Auftraggeber / das Management am Ende des Projekts.Typischerweise wird jeder Projektmanagement-Bereich (Qualität, Kosten, Zeit) mit mindestems einem Ziel belegt. Die Anzahl der Ziele und der Detaillierungsgrad sind eher gering (Management-Kompatibilität!), wo notwendig können Unterdokumente wie z.B. das Pflichtenheft referenziert werden.</t>
-  </si>
-  <si>
-    <t>Zugzielanzeiger</t>
-  </si>
-  <si>
-    <t>Stromversorgung der ZZA</t>
-  </si>
-  <si>
-    <t>Ansteuerung der LED-Matrix</t>
-  </si>
-  <si>
-    <t>Spannungsversorgung an den Netzteilen</t>
-  </si>
-  <si>
-    <t>Teilfunktion 4</t>
-  </si>
-  <si>
-    <t>Getrennte Erdung und Nulleiter</t>
-  </si>
-  <si>
-    <t>Durchgängigkeit des Schutzleiters</t>
-  </si>
-  <si>
-    <t>Einzelne LEDs ansteuerbar</t>
-  </si>
-  <si>
-    <t>Kein erkennbares Flackern der LEDs</t>
-  </si>
-  <si>
-    <t>Anforderung 4</t>
-  </si>
-  <si>
-    <t>Anforderung 5</t>
-  </si>
-  <si>
-    <t>Alle 3 Farben (rot/grün, rot+grün) nutzen</t>
-  </si>
-  <si>
-    <t>Stromversorgung für alle Bauteile des ZZA. Soll sicher sein, dass niemand zu schaden kommt.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Das Pflichtenheft beschreibt alle technischen Eigenschaften des zu entwickelnden Produkts und ist daher typischerweise recht umfangreich. Um den Aufwand im Lernprojekt klein zu halten, soll ein reduziertes Dokument erstellt werden, an dem die Arbeit mit dem Pflichtenheft exemplarisch durchgeführt wird:
-1. Identifizieren Sie die drei wichtigsten Teilfunktionen Ihres ZZA. Definieren Sie für jede dieser drei Teilfunktionen die quantitativen Anforderungen, an denen die technische Zielerreichung gemessen wird. 
-Aus einem guten Pflichtenheft ergibt ich quasi automatisch ein Plan für den Labortest, in dem die Erreichung der technischen Ziele nachgewiesen wird. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Higher level control über die LED-Matrix </t>
-  </si>
-  <si>
-    <t>MCU/FPGA mit 5V TTL und genug Schreibgeschwindigkeit</t>
-  </si>
-  <si>
-    <t>Komplettes Spiel</t>
-  </si>
-  <si>
-    <t>schnelle Ausführung des Codes</t>
-  </si>
-  <si>
-    <t>Eingabegeräte (HID/PC)</t>
-  </si>
-  <si>
-    <t>Nutzen von Controller / Tastatur / Maus um elemente auf dem Display zu steuern. Datenübertragung vom PC aus (mit UART?)</t>
-  </si>
-  <si>
-    <t>Simples Spiel, wie z.B. Pong auf dem ZZA spielen können</t>
-  </si>
-  <si>
-    <t>möglichst kleines Input Delay</t>
-  </si>
-  <si>
-    <t>Ein simples Spiel auf der ZZA laufen lassen, evtl. Zweispieler?</t>
-  </si>
-  <si>
-    <t>Kontrollierte Anzeigen durch LEDs, mit verschiedenen Farben und einer hohen Aktualisierungsrate um Flackern der LEDs zu verhindern.
-Higher level control über die LED-Matrix (Funktionen um z.B. Rechtecke/Linien/etc. anzuzeigen), ganze Reihen/Sektionen ansteuern</t>
+    <t>Risiko</t>
+  </si>
+  <si>
+    <t>Eintritts-
+wahrscheinlichkeit</t>
+  </si>
+  <si>
+    <t>Minderung des  Zielerreichungsgrades bei Risikoeintritt</t>
+  </si>
+  <si>
+    <t>Relevanz des Risikos</t>
+  </si>
+  <si>
+    <t>Gegenmaßnahme</t>
+  </si>
+  <si>
+    <t>erledigt bis</t>
   </si>
   <si>
     <t>Zugzielanzeige Komponenten durchbrennen lassen</t>
@@ -271,24 +268,6 @@
     <t>1-5%</t>
   </si>
   <si>
-    <t>Mai</t>
-  </si>
-  <si>
-    <t>Juni</t>
-  </si>
-  <si>
-    <t>Juli</t>
-  </si>
-  <si>
-    <t>August</t>
-  </si>
-  <si>
-    <t>September</t>
-  </si>
-  <si>
-    <t>alle</t>
-  </si>
-  <si>
     <t>Klausurenphase</t>
   </si>
   <si>
@@ -310,27 +289,9 @@
     <t>nicht funktionierende Eingabegeräte</t>
   </si>
   <si>
-    <t>Rollo die Dampfwalze</t>
-  </si>
-  <si>
-    <t>Mixi der Betonmischer</t>
-  </si>
-  <si>
-    <t>Heppo der Kran</t>
-  </si>
-  <si>
-    <t>Buddel der Schauffellader</t>
-  </si>
-  <si>
-    <t>ZZA reparieren</t>
-  </si>
-  <si>
     <t>Einhaltung der 5 Sicherheitsregeln</t>
   </si>
   <si>
-    <t>Festgurten der ZZA</t>
-  </si>
-  <si>
     <t>Herunterfallen/Umkippen des ZZA</t>
   </si>
   <si>
@@ -343,9 +304,6 @@
     <t>MCU zu langsam</t>
   </si>
   <si>
-    <t>Testen verschiedener MCUs</t>
-  </si>
-  <si>
     <t>Pflichtenhefterfüllung</t>
   </si>
   <si>
@@ -358,29 +316,125 @@
     <t>Risikos</t>
   </si>
   <si>
-    <t>Spaß</t>
-  </si>
-  <si>
     <t>Gesamtausgaben kleiner gleich der Plankosten halten</t>
   </si>
   <si>
-    <t>Gute Zusammenarbeit und PIZZA</t>
-  </si>
-  <si>
-    <t>flexible Teams</t>
-  </si>
-  <si>
-    <t>Jeder hilft jedem</t>
-  </si>
-  <si>
     <t>Erreichung von mindestens 90% der Pflichtenheftforderungen</t>
+  </si>
+  <si>
+    <t>Alle 3 Farben (rot/grün, rot+grün) nutzbar</t>
+  </si>
+  <si>
+    <t>MCU/FPGA mit 5V TTL</t>
+  </si>
+  <si>
+    <t>Input Delay &lt;= 40ms</t>
+  </si>
+  <si>
+    <t>100Hz Abtastrate des Eingabegeräts</t>
+  </si>
+  <si>
+    <t>Simples Spiel (2D-Grafik, 200x64 Pixel Auflösung), wie z.B. Pong auf dem ZZA spielen können</t>
+  </si>
+  <si>
+    <t>schnelle Ausführung des Codes, min. 100Hz Bildwiederholrate</t>
+  </si>
+  <si>
+    <t>Gute Zusammenarbeit</t>
+  </si>
+  <si>
+    <t>Regelmäßige Kommuniktaion</t>
+  </si>
+  <si>
+    <t>min. 90% Teilnahme an den Treffen</t>
+  </si>
+  <si>
+    <t>alle 14 Tage ein Treffen</t>
+  </si>
+  <si>
+    <t>Regelmäßige Dokumentation</t>
+  </si>
+  <si>
+    <t>spätestens 2 Tage nach einem Treffen</t>
+  </si>
+  <si>
+    <t>LED-Matrix kann komplett angesteuert werden</t>
+  </si>
+  <si>
+    <t>Erstes Bild/Frame auf der Matrix</t>
+  </si>
+  <si>
+    <t>Eingabe funktioniert</t>
+  </si>
+  <si>
+    <t>Spiel läuft vollständig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">alle </t>
+  </si>
+  <si>
+    <t>LED-Matrix ansteuern</t>
+  </si>
+  <si>
+    <t>Finn</t>
+  </si>
+  <si>
+    <t>Jan, Mikko</t>
+  </si>
+  <si>
+    <t>Spiel Programmierung</t>
+  </si>
+  <si>
+    <t>Jonas</t>
+  </si>
+  <si>
+    <t>Projektabgabe / Abschlusspräsentation</t>
+  </si>
+  <si>
+    <t>Dokumentation</t>
+  </si>
+  <si>
+    <t>Erik</t>
+  </si>
+  <si>
+    <t>Jan</t>
+  </si>
+  <si>
+    <t>Istkosten [€]*</t>
+  </si>
+  <si>
+    <t>* Beschaffung über uns, keine Kostenübernahme seitens der HAW</t>
+  </si>
+  <si>
+    <t>Jan, Mikko, Finn</t>
+  </si>
+  <si>
+    <t>Finn, Erik</t>
+  </si>
+  <si>
+    <t>Spannungen vor Anschluss überprüfen
+Schaltungen gegenprüfen vor dem Anschließen</t>
+  </si>
+  <si>
+    <t>Stabile Unterkonstruktion
+Festgurten der ZZA</t>
+  </si>
+  <si>
+    <t>Testen verschiedener MCUs
+Prototypen der LED Ansteuerung testen</t>
+  </si>
+  <si>
+    <t>vor Beginn an Arbeiten an der Stromversorgung</t>
+  </si>
+  <si>
+    <t>Vor dem ersten einschalten der Hardware</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -447,6 +501,12 @@
       <i/>
       <sz val="10"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -819,7 +879,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="120">
+  <cellXfs count="125">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -848,6 +908,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -856,9 +919,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -920,9 +980,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1000,9 +1057,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1010,9 +1064,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1041,6 +1092,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -1048,6 +1102,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1057,14 +1114,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1073,6 +1127,33 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -1106,29 +1187,23 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1153,18 +1228,18 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>2</xdr:row>
+      <xdr:row>3</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>3</xdr:row>
+      <xdr:row>4</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="93" name="Abgerundetes Rechteck 2">
+        <xdr:cNvPr id="536" name="Abgerundetes Rechteck 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000003000000}"/>
@@ -1175,8 +1250,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="361950" y="3514724"/>
-          <a:ext cx="1790700" cy="2019301"/>
+          <a:off x="1386417" y="2169582"/>
+          <a:ext cx="1386416" cy="1513417"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
@@ -1345,18 +1420,18 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>2</xdr:row>
+      <xdr:row>3</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>3</xdr:row>
+      <xdr:row>4</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="184" name="Abgerundetes Rechteck 3">
+        <xdr:cNvPr id="535" name="Abgerundetes Rechteck 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000004000000}"/>
@@ -1367,8 +1442,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2533650" y="3524250"/>
-          <a:ext cx="1790700" cy="2009775"/>
+          <a:off x="2714625" y="3529013"/>
+          <a:ext cx="1919288" cy="2009775"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
@@ -1397,11 +1472,11 @@
           <a:pPr algn="l"/>
           <a:r>
             <a:rPr lang="de-DE" sz="1200" b="1"/>
-            <a:t>Erik</a:t>
+            <a:t>Finn</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="de-DE" sz="1200" b="1" baseline="0"/>
-            <a:t> Bröcker</a:t>
+            <a:t> Meister</a:t>
           </a:r>
           <a:endParaRPr lang="de-DE" sz="1200" b="1"/>
         </a:p>
@@ -1513,18 +1588,18 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>2</xdr:row>
+      <xdr:row>3</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>3</xdr:row>
+      <xdr:row>4</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="292" name="Abgerundetes Rechteck 4">
+        <xdr:cNvPr id="562" name="Abgerundetes Rechteck 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000005000000}"/>
@@ -1699,18 +1774,18 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>2</xdr:row>
+      <xdr:row>3</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>3</xdr:row>
+      <xdr:row>4</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="356" name="Abgerundetes Rechteck 5">
+        <xdr:cNvPr id="565" name="Abgerundetes Rechteck 5">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000006000000}"/>
@@ -1897,20 +1972,20 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1076325</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>22410</xdr:rowOff>
+      <xdr:rowOff>212910</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>11204</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>695325</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>2211479</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="454" name="Abgerundetes Rechteck 7">
+        <xdr:cNvPr id="564" name="Abgerundetes Rechteck 7">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000008000000}"/>
@@ -1921,8 +1996,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9054353" y="3552263"/>
-          <a:ext cx="1792941" cy="1994647"/>
+          <a:off x="3609975" y="1060635"/>
+          <a:ext cx="1790700" cy="1998569"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
@@ -1951,11 +2026,7 @@
           <a:pPr algn="l"/>
           <a:r>
             <a:rPr lang="de-DE" sz="1200" b="1"/>
-            <a:t>Finn</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="de-DE" sz="1200" b="1" baseline="0"/>
-            <a:t> Meister</a:t>
+            <a:t>Erik Bröcker</a:t>
           </a:r>
           <a:br>
             <a:rPr lang="de-DE" sz="1200"/>
@@ -2008,19 +2079,19 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>575168</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>23000</xdr:rowOff>
+      <xdr:colOff>621150</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>9862</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>719808</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>195460</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>10359</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>182322</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="26" name="Raute 1">
+        <xdr:cNvPr id="52" name="Raute 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000002000000}"/>
@@ -2031,7 +2102,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="8187841" y="3422692"/>
+          <a:off x="8615581" y="4194293"/>
           <a:ext cx="144640" cy="172460"/>
         </a:xfrm>
         <a:prstGeom prst="diamond">
@@ -2088,7 +2159,7 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="16" name="Abgerundetes Rechteck 3">
+        <xdr:cNvPr id="6" name="Abgerundetes Rechteck 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000004000000}"/>
@@ -2149,7 +2220,7 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="17" name="Abgerundetes Rechteck 3">
+        <xdr:cNvPr id="9" name="Abgerundetes Rechteck 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C7A70151-AE68-4FB7-A006-9124ECC9FA23}"/>
@@ -2198,19 +2269,19 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>432289</xdr:colOff>
-      <xdr:row>13</xdr:row>
+      <xdr:colOff>271463</xdr:colOff>
+      <xdr:row>19</xdr:row>
       <xdr:rowOff>8659</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>743350</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>190500</xdr:rowOff>
+      <xdr:colOff>704850</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>195262</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="22" name="Abgerundetes Rechteck 3">
+        <xdr:cNvPr id="8" name="Abgerundetes Rechteck 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{618BB318-8932-48FA-9C86-92A9FCA7FD11}"/>
@@ -2221,8 +2292,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="8044962" y="3012697"/>
-          <a:ext cx="311061" cy="181841"/>
+          <a:off x="8424863" y="3028084"/>
+          <a:ext cx="433387" cy="186603"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
@@ -2259,19 +2330,19 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>395655</xdr:colOff>
+      <xdr:colOff>454776</xdr:colOff>
       <xdr:row>9</xdr:row>
-      <xdr:rowOff>5004</xdr:rowOff>
+      <xdr:rowOff>11573</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>51288</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>193123</xdr:rowOff>
+      <xdr:colOff>32846</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>2623</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="19" name="Abgerundetes Rechteck 3">
+        <xdr:cNvPr id="65" name="Abgerundetes Rechteck 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{586DF4B5-143F-4CBC-93A9-8EA75A11144F}"/>
@@ -2282,8 +2353,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5788270" y="2217735"/>
-          <a:ext cx="783980" cy="188119"/>
+          <a:off x="6228897" y="2225314"/>
+          <a:ext cx="707932" cy="188119"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
@@ -2332,7 +2403,7 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="25" name="Raute 1">
+        <xdr:cNvPr id="35" name="Raute 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{90B57C9B-D49A-411B-B728-40FC10AA08E2}"/>
@@ -2387,20 +2458,20 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>11</xdr:row>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>523875</xdr:colOff>
+      <xdr:row>14</xdr:row>
       <xdr:rowOff>3538</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>424312</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>191657</xdr:rowOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>195263</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="27" name="Abgerundetes Rechteck 3">
+        <xdr:cNvPr id="5" name="Abgerundetes Rechteck 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7DE4177F-6F29-4C05-9D1A-1B730C3BCCA1}"/>
@@ -2414,8 +2485,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7334250" y="2611923"/>
-          <a:ext cx="702735" cy="188119"/>
+          <a:off x="7515225" y="2622913"/>
+          <a:ext cx="1062487" cy="191725"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
@@ -2458,81 +2529,20 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>512884</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>10865</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>278424</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>1157</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="28" name="Abgerundetes Rechteck 3">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{69EF249E-73B2-405C-8181-8D2A5ECA9222}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="7033846" y="2421423"/>
-          <a:ext cx="293078" cy="188119"/>
-        </a:xfrm>
-        <a:prstGeom prst="roundRect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="12700"/>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1">
-            <a:shade val="50000"/>
-          </a:schemeClr>
-        </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:endParaRPr lang="de-DE" sz="1100"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>322384</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>199899</xdr:rowOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>200024</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>152400</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>185795</xdr:rowOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>185794</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="50" name="Abgerundetes Rechteck 3">
+        <xdr:cNvPr id="66" name="Abgerundetes Rechteck 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{447F8F86-1A35-48C6-9CD9-B216E90798E2}"/>
@@ -2546,8 +2556,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6265984" y="2428749"/>
-          <a:ext cx="411041" cy="185921"/>
+          <a:off x="6646984" y="2628899"/>
+          <a:ext cx="411041" cy="185795"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
@@ -2585,18 +2595,18 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>181841</xdr:colOff>
-      <xdr:row>17</xdr:row>
+      <xdr:row>23</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>514983</xdr:colOff>
-      <xdr:row>17</xdr:row>
+      <xdr:row>23</xdr:row>
       <xdr:rowOff>189451</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="31" name="Abgerundetes Rechteck 3">
+        <xdr:cNvPr id="67" name="Abgerundetes Rechteck 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C0279A3A-CB76-45C8-921E-FB2BB84DAB8C}"/>
@@ -2642,6 +2652,417 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>291620</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>14791</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>442255</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>187251</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="11" name="Raute 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DE5F115B-4266-4BC8-B6ED-48DEDD44BAB1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8286051" y="3410946"/>
+          <a:ext cx="150635" cy="172460"/>
+        </a:xfrm>
+        <a:prstGeom prst="diamond">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="tx1"/>
+        </a:solidFill>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="de-DE" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>206222</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>8223</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>356857</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>180683</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="12" name="Raute 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EF9952D3-5BCD-45AF-A3F9-BE598B70AEC7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6532136" y="2419033"/>
+          <a:ext cx="150635" cy="172460"/>
+        </a:xfrm>
+        <a:prstGeom prst="diamond">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="tx1"/>
+        </a:solidFill>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="de-DE" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>558361</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>13138</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>130927</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>185598</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="14" name="Raute 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0EAA28A1-79E9-4172-8995-6F2033D188DE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6884275" y="3015155"/>
+          <a:ext cx="150635" cy="172460"/>
+        </a:xfrm>
+        <a:prstGeom prst="diamond">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="tx1"/>
+        </a:solidFill>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="de-DE" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>561272</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>19968</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>705912</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>192428</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="15" name="Raute 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4220C93B-7736-477A-A068-8C857A2D9A08}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8555703" y="4007330"/>
+          <a:ext cx="144640" cy="172460"/>
+        </a:xfrm>
+        <a:prstGeom prst="diamond">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="tx1"/>
+        </a:solidFill>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="de-DE" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>480847</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>14452</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>53413</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>186912</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="16" name="Raute 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8A84BCB3-9F8E-42F4-92CB-AA8C80A0D79F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6806761" y="2622331"/>
+          <a:ext cx="150635" cy="172460"/>
+        </a:xfrm>
+        <a:prstGeom prst="diamond">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="tx1"/>
+        </a:solidFill>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="de-DE" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>6897</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>8464</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>748862</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>3120</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="17" name="Abgerundetes Rechteck 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CEDAA15D-757C-4124-B00E-629803B91B55}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{90B57C9B-D49A-411B-B728-40FC10AA08E2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5781018" y="3798757"/>
+          <a:ext cx="2962275" cy="191725"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="12700"/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr marL="0" indent="0" algn="l"/>
+          <a:endParaRPr lang="en-US" sz="1100">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-lt"/>
+            <a:cs typeface="+mn-lt"/>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -2650,15 +3071,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>104775</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
+      <xdr:colOff>66675</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>733425</xdr:colOff>
-      <xdr:row>35</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
+      <xdr:colOff>785812</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2681,7 +3102,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="104775" y="4371975"/>
+          <a:off x="66675" y="4886325"/>
           <a:ext cx="4572000" cy="3257550"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2692,6 +3113,10 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2984,7 +3409,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr defaultColWidth="11.3984375" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="86.1328125" style="3" customWidth="1"/>
@@ -2994,185 +3419,193 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.65">
-      <c r="A1" s="103" t="s">
-        <v>11</v>
-      </c>
-      <c r="B1" s="104"/>
-      <c r="C1" s="14"/>
+      <c r="A1" s="110" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="111"/>
+      <c r="C1" s="15"/>
     </row>
     <row r="2" spans="1:6" ht="61.9" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="101" t="s">
-        <v>46</v>
-      </c>
-      <c r="B2" s="102"/>
-      <c r="C2" s="102"/>
+      <c r="A2" s="108" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="109"/>
+      <c r="C2" s="109"/>
     </row>
     <row r="3" spans="1:6" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A3" s="17" t="s">
-        <v>38</v>
-      </c>
-      <c r="B3" s="40" t="s">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="B3" s="39" t="s">
+        <v>3</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>39</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A4" s="19" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" s="41"/>
+        <v>5</v>
+      </c>
+      <c r="B4" s="40"/>
       <c r="C4" s="21"/>
     </row>
     <row r="5" spans="1:6" ht="31.5" x14ac:dyDescent="0.45">
-      <c r="A5" s="48" t="s">
+      <c r="A5" s="47" t="s">
+        <v>83</v>
+      </c>
+      <c r="B5" s="42">
+        <v>2</v>
+      </c>
+      <c r="C5" s="45" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="15.75" x14ac:dyDescent="0.45">
+      <c r="A6" s="43"/>
+      <c r="B6" s="41"/>
+      <c r="C6" s="45"/>
+    </row>
+    <row r="7" spans="1:6" ht="15.75" x14ac:dyDescent="0.45">
+      <c r="A7" s="46" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="42"/>
+      <c r="C7" s="45"/>
+      <c r="D7" s="38"/>
+    </row>
+    <row r="8" spans="1:6" ht="47.25" x14ac:dyDescent="0.45">
+      <c r="A8" s="47" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8" s="42">
+        <v>3</v>
+      </c>
+      <c r="C8" s="45" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="15.75" x14ac:dyDescent="0.45">
+      <c r="A9" s="43"/>
+      <c r="B9" s="41"/>
+      <c r="C9" s="44"/>
+    </row>
+    <row r="10" spans="1:6" ht="15.75" x14ac:dyDescent="0.45">
+      <c r="A10" s="46" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" s="42"/>
+      <c r="C10" s="45"/>
+    </row>
+    <row r="11" spans="1:6" ht="31.5" x14ac:dyDescent="0.45">
+      <c r="A11" s="47" t="s">
+        <v>84</v>
+      </c>
+      <c r="B11" s="42">
+        <v>4</v>
+      </c>
+      <c r="C11" s="45" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="15.75" x14ac:dyDescent="0.45">
+      <c r="A12" s="47"/>
+      <c r="B12" s="42"/>
+      <c r="C12" s="45"/>
+    </row>
+    <row r="13" spans="1:6" ht="15.75" x14ac:dyDescent="0.45">
+      <c r="A13" s="46" t="s">
+        <v>10</v>
+      </c>
+      <c r="B13" s="40"/>
+      <c r="C13" s="48"/>
+    </row>
+    <row r="14" spans="1:6" ht="15.75" x14ac:dyDescent="0.45">
+      <c r="A14" s="47" t="s">
+        <v>95</v>
+      </c>
+      <c r="B14" s="42">
+        <v>1</v>
+      </c>
+      <c r="C14" s="45" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="15.75" x14ac:dyDescent="0.45">
+      <c r="A15" s="47" t="s">
+        <v>96</v>
+      </c>
+      <c r="B15" s="42">
+        <v>1</v>
+      </c>
+      <c r="C15" s="45" t="s">
         <v>98</v>
       </c>
-      <c r="B5" s="43">
-        <v>2</v>
-      </c>
-      <c r="C5" s="46" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="15.75" x14ac:dyDescent="0.45">
-      <c r="A6" s="44"/>
-      <c r="B6" s="42"/>
-      <c r="C6" s="46"/>
-    </row>
-    <row r="7" spans="1:6" ht="15.75" x14ac:dyDescent="0.45">
-      <c r="A7" s="47" t="s">
-        <v>19</v>
-      </c>
-      <c r="B7" s="43"/>
-      <c r="C7" s="46"/>
-      <c r="D7" s="39"/>
-    </row>
-    <row r="8" spans="1:6" ht="47.25" x14ac:dyDescent="0.45">
-      <c r="A8" s="48" t="s">
-        <v>24</v>
-      </c>
-      <c r="B8" s="43">
-        <v>3</v>
-      </c>
-      <c r="C8" s="46" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="15.75" x14ac:dyDescent="0.45">
-      <c r="A9" s="44"/>
-      <c r="B9" s="42"/>
-      <c r="C9" s="45"/>
-    </row>
-    <row r="10" spans="1:6" ht="15.75" x14ac:dyDescent="0.45">
-      <c r="A10" s="47" t="s">
-        <v>20</v>
-      </c>
-      <c r="B10" s="43"/>
-      <c r="C10" s="46"/>
-    </row>
-    <row r="11" spans="1:6" ht="31.5" x14ac:dyDescent="0.45">
-      <c r="A11" s="48" t="s">
+      <c r="F15" s="95"/>
+    </row>
+    <row r="16" spans="1:6" ht="15.75" x14ac:dyDescent="0.45">
+      <c r="A16" s="47" t="s">
         <v>99</v>
       </c>
-      <c r="B11" s="43">
-        <v>4</v>
-      </c>
-      <c r="C11" s="46" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="15.75" x14ac:dyDescent="0.45">
-      <c r="A12" s="48"/>
-      <c r="B12" s="43"/>
-      <c r="C12" s="46"/>
-    </row>
-    <row r="13" spans="1:6" ht="15.75" x14ac:dyDescent="0.45">
-      <c r="A13" s="47" t="s">
-        <v>21</v>
-      </c>
-      <c r="B13" s="41"/>
-      <c r="C13" s="49"/>
-    </row>
-    <row r="14" spans="1:6" ht="15.75" x14ac:dyDescent="0.45">
-      <c r="A14" s="48" t="s">
-        <v>102</v>
-      </c>
-      <c r="B14" s="43">
+      <c r="B16" s="42">
         <v>1</v>
       </c>
-      <c r="C14" s="46" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="15.75" x14ac:dyDescent="0.45">
-      <c r="A15" s="48" t="s">
-        <v>105</v>
-      </c>
-      <c r="B15" s="43">
-        <v>1</v>
-      </c>
-      <c r="C15" s="46" t="s">
-        <v>106</v>
-      </c>
-      <c r="F15" s="96"/>
-    </row>
-    <row r="16" spans="1:6" ht="15.75" x14ac:dyDescent="0.45">
-      <c r="A16" s="48"/>
-      <c r="B16" s="43"/>
-      <c r="C16" s="46"/>
-      <c r="F16" s="96"/>
+      <c r="C16" s="45" t="s">
+        <v>100</v>
+      </c>
+      <c r="F16" s="95"/>
     </row>
     <row r="17" spans="1:6" ht="15.75" x14ac:dyDescent="0.45">
-      <c r="A17" s="47" t="s">
-        <v>22</v>
-      </c>
-      <c r="B17" s="41"/>
-      <c r="C17" s="49"/>
+      <c r="A17" s="47"/>
+      <c r="B17" s="42"/>
+      <c r="C17" s="45"/>
+      <c r="F17" s="95"/>
     </row>
     <row r="18" spans="1:6" ht="15.75" x14ac:dyDescent="0.45">
-      <c r="A18" s="48" t="s">
-        <v>101</v>
-      </c>
-      <c r="B18" s="43">
+      <c r="A18" s="46" t="s">
+        <v>11</v>
+      </c>
+      <c r="B18" s="40"/>
+      <c r="C18" s="48"/>
+    </row>
+    <row r="19" spans="1:6" ht="15.75" x14ac:dyDescent="0.45">
+      <c r="A19" s="47" t="s">
+        <v>86</v>
+      </c>
+      <c r="B19" s="42">
         <v>0</v>
       </c>
-      <c r="C18" s="46" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="15.75" x14ac:dyDescent="0.45">
-      <c r="A19" s="44"/>
-      <c r="B19" s="42"/>
-      <c r="C19" s="45"/>
-    </row>
-    <row r="20" spans="1:6" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A20" s="24"/>
-      <c r="B20" s="23"/>
-      <c r="C20" s="22"/>
+      <c r="C19" s="45" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="15.75" x14ac:dyDescent="0.45">
+      <c r="A20" s="43"/>
+      <c r="B20" s="41"/>
+      <c r="C20" s="44"/>
     </row>
     <row r="21" spans="1:6" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A21" s="25"/>
-      <c r="B21" s="26"/>
-      <c r="C21" s="27"/>
+      <c r="A21" s="24"/>
+      <c r="B21" s="23"/>
+      <c r="C21" s="22"/>
     </row>
     <row r="22" spans="1:6" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A22" s="28"/>
-      <c r="B22" s="29"/>
-      <c r="C22" s="30"/>
-      <c r="E22" s="97"/>
-    </row>
-    <row r="23" spans="1:6" ht="24.4" x14ac:dyDescent="0.85">
-      <c r="A23" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="B23" s="20"/>
-      <c r="C23" s="98"/>
+      <c r="A22" s="25"/>
+      <c r="B22" s="26"/>
+      <c r="C22" s="27"/>
+    </row>
+    <row r="23" spans="1:6" ht="15.75" x14ac:dyDescent="0.5">
+      <c r="A23" s="28"/>
+      <c r="B23" s="29"/>
+      <c r="C23" s="30"/>
+      <c r="E23" s="96"/>
     </row>
     <row r="24" spans="1:6" ht="24.4" x14ac:dyDescent="0.85">
+      <c r="A24" s="19" t="s">
+        <v>12</v>
+      </c>
       <c r="B24" s="20"/>
-      <c r="C24" s="99"/>
+      <c r="C24" s="97"/>
     </row>
     <row r="25" spans="1:6" ht="24.4" x14ac:dyDescent="0.85">
       <c r="B25" s="20"/>
@@ -3180,38 +3613,42 @@
     </row>
     <row r="26" spans="1:6" ht="24.4" x14ac:dyDescent="0.85">
       <c r="B26" s="20"/>
-      <c r="C26" s="100"/>
-      <c r="F26" s="97"/>
+      <c r="C26" s="97"/>
     </row>
     <row r="27" spans="1:6" ht="24.4" x14ac:dyDescent="0.85">
-      <c r="A27" s="19"/>
       <c r="B27" s="20"/>
-      <c r="C27" s="98"/>
-    </row>
-    <row r="28" spans="1:6" ht="15.75" x14ac:dyDescent="0.5">
+      <c r="C27" s="99"/>
+      <c r="F27" s="96"/>
+    </row>
+    <row r="28" spans="1:6" ht="24.4" x14ac:dyDescent="0.85">
       <c r="A28" s="19"/>
       <c r="B28" s="20"/>
-      <c r="C28" s="22"/>
+      <c r="C28" s="97"/>
     </row>
     <row r="29" spans="1:6" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A29" s="19" t="s">
-        <v>15</v>
-      </c>
+      <c r="A29" s="19"/>
       <c r="B29" s="20"/>
       <c r="C29" s="22"/>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A30" s="5"/>
-      <c r="C30" s="4"/>
+    <row r="30" spans="1:6" ht="15.75" x14ac:dyDescent="0.5">
+      <c r="A30" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="B30" s="20"/>
+      <c r="C30" s="22"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A31" s="5"/>
       <c r="C31" s="4"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A32" s="6"/>
-      <c r="B32" s="9"/>
-      <c r="C32" s="7"/>
+      <c r="A32" s="5"/>
+      <c r="C32" s="4"/>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A33" s="6"/>
+      <c r="B33" s="9"/>
+      <c r="C33" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3229,213 +3666,216 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B1:C33"/>
-  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="11.3984375" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="4.1328125" customWidth="1"/>
     <col min="2" max="2" width="40" customWidth="1"/>
     <col min="3" max="3" width="52.265625" style="8" customWidth="1"/>
+    <col min="4" max="4" width="11.3984375" customWidth="1"/>
     <col min="6" max="6" width="80.73046875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:3" ht="21" x14ac:dyDescent="0.65">
-      <c r="B1" s="105" t="s">
-        <v>13</v>
-      </c>
-      <c r="C1" s="106"/>
+      <c r="B1" s="112" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="113"/>
     </row>
     <row r="2" spans="2:3" ht="112.9" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B2" s="107" t="s">
-        <v>60</v>
-      </c>
-      <c r="C2" s="108"/>
+      <c r="B2" s="114" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="115"/>
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.45">
       <c r="B4" s="9"/>
-      <c r="C4" s="15"/>
+      <c r="C4" s="16"/>
     </row>
     <row r="5" spans="2:3" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="B5" s="50" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" s="51" t="s">
-        <v>48</v>
+      <c r="B5" s="49" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="50" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="2:3" ht="105.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B6" s="52" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" s="55" t="s">
-        <v>59</v>
+      <c r="B6" s="51" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="54" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="7" spans="2:3" ht="15.75" x14ac:dyDescent="0.5">
       <c r="B7" s="19" t="s">
-        <v>2</v>
-      </c>
-      <c r="C7" s="78" t="s">
-        <v>52</v>
+        <v>20</v>
+      </c>
+      <c r="C7" s="75" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="2:3" ht="15.75" x14ac:dyDescent="0.5">
       <c r="B8" s="19" t="s">
-        <v>4</v>
-      </c>
-      <c r="C8" s="56" t="s">
-        <v>50</v>
+        <v>22</v>
+      </c>
+      <c r="C8" s="55" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="9" spans="2:3" ht="15.75" x14ac:dyDescent="0.5">
       <c r="B9" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="C9" s="56" t="s">
-        <v>53</v>
+        <v>24</v>
+      </c>
+      <c r="C9" s="55" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="2:3" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="B10" s="53"/>
-      <c r="C10" s="54"/>
+      <c r="B10" s="52"/>
+      <c r="C10" s="53"/>
     </row>
     <row r="11" spans="2:3" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="B11" s="50" t="s">
-        <v>16</v>
-      </c>
-      <c r="C11" s="51" t="s">
-        <v>49</v>
+      <c r="B11" s="49" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" s="50" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="12" spans="2:3" ht="113.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B12" s="52" t="s">
-        <v>5</v>
-      </c>
-      <c r="C12" s="55" t="s">
-        <v>70</v>
+      <c r="B12" s="51" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="54" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="13" spans="2:3" ht="15.75" x14ac:dyDescent="0.5">
       <c r="B13" s="19" t="s">
-        <v>2</v>
-      </c>
-      <c r="C13" s="56" t="s">
-        <v>55</v>
+        <v>20</v>
+      </c>
+      <c r="C13" s="55" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="14" spans="2:3" ht="15.75" x14ac:dyDescent="0.5">
       <c r="B14" s="19" t="s">
-        <v>4</v>
-      </c>
-      <c r="C14" s="56" t="s">
-        <v>54</v>
+        <v>22</v>
+      </c>
+      <c r="C14" s="55" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="15" spans="2:3" ht="15.75" x14ac:dyDescent="0.5">
       <c r="B15" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="C15" s="56" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="16" spans="2:3" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.5">
+        <v>24</v>
+      </c>
+      <c r="C15" s="55" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="16" spans="2:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B16" s="19" t="s">
-        <v>56</v>
-      </c>
-      <c r="C16" s="56" t="s">
-        <v>62</v>
+        <v>31</v>
+      </c>
+      <c r="C16" s="55" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="17" spans="2:3" ht="15.75" x14ac:dyDescent="0.5">
       <c r="B17" s="19" t="s">
-        <v>57</v>
-      </c>
-      <c r="C17" s="76" t="s">
-        <v>61</v>
+        <v>32</v>
+      </c>
+      <c r="C17" s="54" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="18" spans="2:3" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="B18" s="57" t="s">
-        <v>12</v>
-      </c>
-      <c r="C18" s="58"/>
+      <c r="B18" s="56" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" s="57"/>
     </row>
     <row r="19" spans="2:3" ht="15.75" x14ac:dyDescent="0.5">
       <c r="B19" s="26"/>
-      <c r="C19" s="59"/>
+      <c r="C19" s="58"/>
     </row>
     <row r="20" spans="2:3" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="B20" s="50" t="s">
-        <v>17</v>
-      </c>
-      <c r="C20" s="51" t="s">
-        <v>65</v>
+      <c r="B20" s="49" t="s">
+        <v>34</v>
+      </c>
+      <c r="C20" s="50" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="21" spans="2:3" ht="105.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B21" s="52" t="s">
-        <v>5</v>
-      </c>
-      <c r="C21" s="55" t="s">
-        <v>66</v>
+      <c r="B21" s="51" t="s">
+        <v>18</v>
+      </c>
+      <c r="C21" s="54" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="22" spans="2:3" ht="15.75" x14ac:dyDescent="0.5">
       <c r="B22" s="19" t="s">
-        <v>2</v>
-      </c>
-      <c r="C22" s="56" t="s">
-        <v>68</v>
+        <v>20</v>
+      </c>
+      <c r="C22" s="55" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="23" spans="2:3" ht="15.75" x14ac:dyDescent="0.5">
       <c r="B23" s="19" t="s">
-        <v>4</v>
-      </c>
-      <c r="C23" s="56"/>
+        <v>22</v>
+      </c>
+      <c r="C23" s="55" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="24" spans="2:3" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="B24" s="57" t="s">
-        <v>12</v>
-      </c>
-      <c r="C24" s="58"/>
+      <c r="B24" s="56" t="s">
+        <v>9</v>
+      </c>
+      <c r="C24" s="57"/>
     </row>
     <row r="26" spans="2:3" ht="15.4" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="B26" s="50" t="s">
-        <v>51</v>
-      </c>
-      <c r="C26" s="51" t="s">
-        <v>63</v>
+      <c r="B26" s="49" t="s">
+        <v>37</v>
+      </c>
+      <c r="C26" s="50" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="27" spans="2:3" ht="94.15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B27" s="52" t="s">
-        <v>5</v>
-      </c>
-      <c r="C27" s="77" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="28" spans="2:3" ht="15.75" x14ac:dyDescent="0.5">
+      <c r="B27" s="51" t="s">
+        <v>18</v>
+      </c>
+      <c r="C27" s="74" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="28" spans="2:3" ht="31.5" x14ac:dyDescent="0.5">
       <c r="B28" s="19" t="s">
-        <v>2</v>
-      </c>
-      <c r="C28" s="55" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="29" spans="2:3" ht="15.75" x14ac:dyDescent="0.5">
+        <v>20</v>
+      </c>
+      <c r="C28" s="54" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="29" spans="2:3" ht="31.5" x14ac:dyDescent="0.5">
       <c r="B29" s="19" t="s">
-        <v>4</v>
-      </c>
-      <c r="C29" s="56" t="s">
-        <v>64</v>
+        <v>22</v>
+      </c>
+      <c r="C29" s="55" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="30" spans="2:3" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="B30" s="57" t="s">
-        <v>12</v>
-      </c>
-      <c r="C30" s="58"/>
+      <c r="B30" s="56" t="s">
+        <v>9</v>
+      </c>
+      <c r="C30" s="57"/>
     </row>
     <row r="33" ht="108.6" customHeight="1" x14ac:dyDescent="0.45"/>
   </sheetData>
@@ -3443,15 +3883,19 @@
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="45" fitToHeight="0" orientation="portrait" r:id="rId1"/>
+  <phoneticPr fontId="9" type="noConversion"/>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:J27"/>
-  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:J28"/>
+  <sheetFormatPr defaultColWidth="11.3984375" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="5.3984375" customWidth="1"/>
     <col min="2" max="2" width="26.86328125" customWidth="1"/>
@@ -3466,46 +3910,57 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.65">
-      <c r="A1" s="103" t="s">
-        <v>28</v>
-      </c>
-      <c r="B1" s="109"/>
-      <c r="C1" s="109"/>
-      <c r="D1" s="109"/>
-      <c r="E1" s="109"/>
-      <c r="F1" s="109"/>
-      <c r="G1" s="109"/>
-      <c r="H1" s="109"/>
-      <c r="I1" s="109"/>
-      <c r="J1" s="110"/>
+      <c r="A1" s="110" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" s="116"/>
+      <c r="C1" s="116"/>
+      <c r="D1" s="116"/>
+      <c r="E1" s="116"/>
+      <c r="F1" s="116"/>
+      <c r="G1" s="116"/>
+      <c r="H1" s="116"/>
+      <c r="I1" s="116"/>
+      <c r="J1" s="117"/>
     </row>
     <row r="2" spans="1:10" ht="46.15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="111" t="s">
-        <v>45</v>
-      </c>
-      <c r="B2" s="112"/>
-      <c r="C2" s="112"/>
-      <c r="D2" s="112"/>
-      <c r="E2" s="112"/>
-      <c r="F2" s="112"/>
-      <c r="G2" s="112"/>
-      <c r="H2" s="112"/>
-      <c r="I2" s="112"/>
-      <c r="J2" s="113"/>
-    </row>
-    <row r="3" spans="1:10" ht="158.25" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A3" s="72"/>
-      <c r="B3" s="73"/>
-      <c r="C3" s="73"/>
-      <c r="D3" s="73"/>
-      <c r="E3" s="73"/>
-      <c r="F3" s="73"/>
-      <c r="G3" s="73"/>
-      <c r="H3" s="73"/>
-      <c r="I3" s="73"/>
-      <c r="J3" s="74"/>
-    </row>
-    <row r="4" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.45"/>
+      <c r="A2" s="118" t="s">
+        <v>41</v>
+      </c>
+      <c r="B2" s="106"/>
+      <c r="C2" s="106"/>
+      <c r="D2" s="106"/>
+      <c r="E2" s="106"/>
+      <c r="F2" s="106"/>
+      <c r="G2" s="106"/>
+      <c r="H2" s="106"/>
+      <c r="I2" s="106"/>
+      <c r="J2" s="119"/>
+    </row>
+    <row r="3" spans="1:10" ht="193.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A3" s="100"/>
+      <c r="B3" s="101"/>
+      <c r="C3" s="101"/>
+      <c r="D3" s="101"/>
+      <c r="E3" s="101"/>
+      <c r="F3" s="101"/>
+      <c r="G3" s="101"/>
+      <c r="H3" s="101"/>
+      <c r="I3" s="101"/>
+      <c r="J3" s="102"/>
+    </row>
+    <row r="4" spans="1:10" ht="158.25" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A4" s="70"/>
+      <c r="B4" s="71"/>
+      <c r="C4" s="71"/>
+      <c r="D4" s="71"/>
+      <c r="E4" s="71"/>
+      <c r="F4" s="71"/>
+      <c r="G4" s="71"/>
+      <c r="H4" s="71"/>
+      <c r="I4" s="71"/>
+      <c r="J4" s="72"/>
+    </row>
     <row r="5" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="6" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="7" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.45"/>
@@ -3529,12 +3984,13 @@
     <row r="25" ht="60" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="26" ht="60" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="27" ht="60" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="28" ht="60" customHeight="1" x14ac:dyDescent="0.45"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
@@ -3545,11 +4001,11 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O39"/>
-  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:O46"/>
+  <sheetFormatPr defaultColWidth="11.3984375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="7.1328125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="43" customWidth="1"/>
+    <col min="2" max="2" width="48.73046875" customWidth="1"/>
     <col min="3" max="3" width="30.73046875" customWidth="1"/>
     <col min="4" max="4" width="8.265625" customWidth="1"/>
     <col min="5" max="5" width="8.73046875" customWidth="1"/>
@@ -3559,564 +4015,662 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="21" x14ac:dyDescent="0.65">
-      <c r="A1" s="114" t="s">
-        <v>24</v>
-      </c>
-      <c r="B1" s="115"/>
-      <c r="C1" s="115"/>
-      <c r="D1" s="115"/>
-      <c r="E1" s="81"/>
-      <c r="F1" s="81"/>
-      <c r="G1" s="81"/>
-      <c r="H1" s="82"/>
+      <c r="A1" s="103" t="s">
+        <v>42</v>
+      </c>
+      <c r="B1" s="104"/>
+      <c r="C1" s="104"/>
+      <c r="D1" s="104"/>
+      <c r="E1" s="78"/>
+      <c r="F1" s="78"/>
+      <c r="G1" s="78"/>
+      <c r="H1" s="79"/>
     </row>
     <row r="2" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="116" t="s">
+      <c r="A2" s="105" t="s">
         <v>43</v>
       </c>
-      <c r="B2" s="112"/>
-      <c r="C2" s="112"/>
-      <c r="D2" s="112"/>
-      <c r="E2" s="112"/>
-      <c r="F2" s="112"/>
-      <c r="G2" s="112"/>
-      <c r="H2" s="117"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A3" s="83"/>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-      <c r="H3" s="12"/>
+      <c r="B2" s="106"/>
+      <c r="C2" s="106"/>
+      <c r="D2" s="106"/>
+      <c r="E2" s="106"/>
+      <c r="F2" s="106"/>
+      <c r="G2" s="106"/>
+      <c r="H2" s="107"/>
+    </row>
+    <row r="3" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A3" s="80"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="13"/>
     </row>
     <row r="4" spans="1:8" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A4" s="84" t="s">
-        <v>25</v>
-      </c>
-      <c r="B4" s="61" t="s">
-        <v>26</v>
-      </c>
-      <c r="C4" s="68" t="s">
-        <v>27</v>
-      </c>
-      <c r="D4" s="80" t="s">
-        <v>73</v>
-      </c>
-      <c r="E4" s="75" t="s">
-        <v>74</v>
-      </c>
-      <c r="F4" s="75" t="s">
-        <v>75</v>
-      </c>
-      <c r="G4" s="75" t="s">
-        <v>76</v>
-      </c>
-      <c r="H4" s="85" t="s">
-        <v>77</v>
+      <c r="A4" s="81" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4" s="60" t="s">
+        <v>45</v>
+      </c>
+      <c r="C4" s="67" t="s">
+        <v>46</v>
+      </c>
+      <c r="D4" s="77" t="s">
+        <v>47</v>
+      </c>
+      <c r="E4" s="73" t="s">
+        <v>48</v>
+      </c>
+      <c r="F4" s="73" t="s">
+        <v>49</v>
+      </c>
+      <c r="G4" s="73" t="s">
+        <v>50</v>
+      </c>
+      <c r="H4" s="82" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:8" s="8" customFormat="1" ht="15.75" x14ac:dyDescent="0.45">
-      <c r="A5" s="86"/>
-      <c r="B5" s="55"/>
-      <c r="C5" s="69"/>
-      <c r="D5" s="70"/>
-      <c r="E5" s="70"/>
-      <c r="F5" s="70"/>
-      <c r="G5" s="70"/>
-      <c r="H5" s="87"/>
+      <c r="A5" s="83"/>
+      <c r="B5" s="54"/>
+      <c r="C5" s="68"/>
+      <c r="D5" s="84"/>
+      <c r="E5" s="84"/>
+      <c r="F5" s="84"/>
+      <c r="G5" s="84"/>
+      <c r="H5" s="85"/>
     </row>
     <row r="6" spans="1:8" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A6" s="88">
+      <c r="A6" s="86">
         <v>1</v>
       </c>
-      <c r="B6" s="63" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" s="71" t="s">
-        <v>78</v>
-      </c>
-      <c r="D6" s="89"/>
-      <c r="E6" s="89"/>
-      <c r="F6" s="89"/>
-      <c r="G6" s="89"/>
-      <c r="H6" s="71"/>
+      <c r="B6" s="62" t="s">
+        <v>52</v>
+      </c>
+      <c r="C6" s="69" t="s">
+        <v>53</v>
+      </c>
+      <c r="D6" s="87"/>
+      <c r="E6" s="87"/>
+      <c r="F6" s="87"/>
+      <c r="G6" s="87"/>
+      <c r="H6" s="69"/>
     </row>
     <row r="7" spans="1:8" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A7" s="88"/>
-      <c r="B7" s="63" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7" s="71" t="s">
-        <v>78</v>
-      </c>
-      <c r="D7" s="89"/>
-      <c r="E7" s="89"/>
-      <c r="F7" s="89"/>
-      <c r="G7" s="89"/>
-      <c r="H7" s="71"/>
+      <c r="A7" s="86"/>
+      <c r="B7" s="62" t="s">
+        <v>54</v>
+      </c>
+      <c r="C7" s="69" t="s">
+        <v>53</v>
+      </c>
+      <c r="D7" s="87"/>
+      <c r="E7" s="87"/>
+      <c r="F7" s="87"/>
+      <c r="G7" s="87"/>
+      <c r="H7" s="69"/>
     </row>
     <row r="8" spans="1:8" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A8" s="88"/>
-      <c r="B8" s="79"/>
-      <c r="C8" s="71"/>
-      <c r="D8" s="89"/>
-      <c r="E8" s="89"/>
-      <c r="F8" s="89"/>
-      <c r="G8" s="89"/>
-      <c r="H8" s="71"/>
+      <c r="B8" s="76"/>
+      <c r="C8" s="69"/>
+      <c r="D8" s="87"/>
+      <c r="E8" s="87"/>
+      <c r="F8" s="87"/>
+      <c r="G8" s="87"/>
+      <c r="H8" s="69"/>
     </row>
     <row r="9" spans="1:8" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A9" s="88"/>
-      <c r="B9" s="63" t="s">
-        <v>48</v>
-      </c>
-      <c r="C9" s="71"/>
-      <c r="D9" s="89"/>
-      <c r="E9" s="89"/>
-      <c r="F9" s="89"/>
-      <c r="G9" s="89"/>
-      <c r="H9" s="71"/>
+      <c r="A9" s="86"/>
+      <c r="B9" s="62" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="69" t="s">
+        <v>108</v>
+      </c>
+      <c r="D9" s="87"/>
+      <c r="E9" s="87"/>
+      <c r="F9" s="87"/>
+      <c r="G9" s="87"/>
+      <c r="H9" s="69"/>
     </row>
     <row r="10" spans="1:8" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A10" s="88"/>
-      <c r="B10" s="63" t="s">
-        <v>49</v>
-      </c>
-      <c r="C10" s="71"/>
-      <c r="D10" s="89"/>
-      <c r="E10" s="89"/>
-      <c r="F10" s="89"/>
-      <c r="G10" s="89"/>
-      <c r="H10" s="71"/>
+      <c r="A10" s="86"/>
+      <c r="B10" s="62" t="s">
+        <v>106</v>
+      </c>
+      <c r="C10" s="69" t="s">
+        <v>107</v>
+      </c>
+      <c r="D10" s="87"/>
+      <c r="E10" s="87"/>
+      <c r="F10" s="87"/>
+      <c r="G10" s="87"/>
+      <c r="H10" s="69"/>
     </row>
     <row r="11" spans="1:8" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A11" s="88"/>
-      <c r="B11" s="63" t="s">
-        <v>65</v>
-      </c>
-      <c r="C11" s="71"/>
-      <c r="D11" s="89"/>
-      <c r="E11" s="89"/>
-      <c r="F11" s="89"/>
-      <c r="G11" s="89"/>
-      <c r="H11" s="71"/>
+      <c r="A11" s="86"/>
+      <c r="B11" s="62" t="s">
+        <v>101</v>
+      </c>
+      <c r="C11" s="69"/>
+      <c r="D11" s="87"/>
+      <c r="E11" s="87"/>
+      <c r="F11" s="87"/>
+      <c r="G11" s="87"/>
+      <c r="H11" s="69"/>
     </row>
     <row r="12" spans="1:8" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A12" s="88"/>
-      <c r="B12" s="63" t="s">
-        <v>63</v>
-      </c>
-      <c r="C12" s="71"/>
-      <c r="D12" s="89"/>
-      <c r="E12" s="89"/>
-      <c r="F12" s="89"/>
-      <c r="G12" s="89"/>
-      <c r="H12" s="71"/>
+      <c r="A12" s="86"/>
+      <c r="B12" s="62" t="s">
+        <v>102</v>
+      </c>
+      <c r="C12" s="69"/>
+      <c r="D12" s="87"/>
+      <c r="E12" s="87"/>
+      <c r="F12" s="87"/>
+      <c r="G12" s="87"/>
+      <c r="H12" s="69"/>
     </row>
     <row r="13" spans="1:8" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A13" s="88"/>
-      <c r="B13" s="63"/>
-      <c r="C13" s="71"/>
-      <c r="D13" s="89"/>
-      <c r="E13" s="89"/>
-      <c r="F13" s="89"/>
-      <c r="G13" s="89"/>
-      <c r="H13" s="71"/>
+      <c r="A13" s="86"/>
+      <c r="B13" s="62" t="s">
+        <v>35</v>
+      </c>
+      <c r="C13" s="69" t="s">
+        <v>114</v>
+      </c>
+      <c r="D13" s="87"/>
+      <c r="E13" s="87"/>
+      <c r="F13" s="87"/>
+      <c r="G13" s="87"/>
+      <c r="H13" s="69"/>
     </row>
     <row r="14" spans="1:8" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A14" s="88"/>
-      <c r="B14" s="63" t="s">
-        <v>9</v>
-      </c>
-      <c r="C14" s="71"/>
-      <c r="D14" s="89"/>
-      <c r="E14" s="89"/>
-      <c r="F14" s="89"/>
-      <c r="G14" s="89"/>
-      <c r="H14" s="71"/>
+      <c r="A14" s="86"/>
+      <c r="B14" s="62" t="s">
+        <v>103</v>
+      </c>
+      <c r="C14" s="69"/>
+      <c r="D14" s="87"/>
+      <c r="E14" s="87"/>
+      <c r="F14" s="87"/>
+      <c r="G14" s="87"/>
+      <c r="H14" s="69"/>
     </row>
     <row r="15" spans="1:8" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A15" s="88"/>
-      <c r="B15" s="63"/>
-      <c r="C15" s="71"/>
-      <c r="D15" s="89"/>
-      <c r="E15" s="89"/>
-      <c r="F15" s="89"/>
-      <c r="G15" s="89"/>
-      <c r="H15" s="71"/>
+      <c r="A15" s="86"/>
+      <c r="B15" s="62" t="s">
+        <v>109</v>
+      </c>
+      <c r="C15" s="69" t="s">
+        <v>110</v>
+      </c>
+      <c r="D15" s="87"/>
+      <c r="E15" s="87"/>
+      <c r="F15" s="87"/>
+      <c r="G15" s="87"/>
+      <c r="H15" s="69"/>
     </row>
     <row r="16" spans="1:8" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A16" s="88"/>
-      <c r="B16" s="63" t="s">
-        <v>10</v>
-      </c>
-      <c r="C16" s="71"/>
-      <c r="D16" s="89"/>
-      <c r="E16" s="89"/>
-      <c r="F16" s="89"/>
-      <c r="G16" s="89"/>
-      <c r="H16" s="71"/>
+      <c r="A16" s="86"/>
+      <c r="B16" s="62" t="s">
+        <v>104</v>
+      </c>
+      <c r="C16" s="69"/>
+      <c r="D16" s="87"/>
+      <c r="E16" s="87"/>
+      <c r="F16" s="87"/>
+      <c r="G16" s="87"/>
+      <c r="H16" s="69"/>
     </row>
     <row r="17" spans="1:15" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A17" s="88"/>
-      <c r="B17" s="63"/>
-      <c r="C17" s="71"/>
-      <c r="D17" s="89"/>
-      <c r="E17" s="89"/>
-      <c r="F17" s="89"/>
-      <c r="G17" s="89"/>
-      <c r="H17" s="71"/>
-      <c r="O17" s="8"/>
+      <c r="A17" s="86"/>
+      <c r="B17" s="62"/>
+      <c r="C17" s="69"/>
+      <c r="D17" s="87"/>
+      <c r="E17" s="87"/>
+      <c r="F17" s="87"/>
+      <c r="G17" s="87"/>
+      <c r="H17" s="69"/>
     </row>
     <row r="18" spans="1:15" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A18" s="88"/>
-      <c r="B18" s="64" t="s">
-        <v>79</v>
-      </c>
-      <c r="C18" s="71"/>
-      <c r="D18" s="89"/>
-      <c r="E18" s="89"/>
-      <c r="F18" s="89"/>
-      <c r="G18" s="89"/>
-      <c r="H18" s="71"/>
+      <c r="A18" s="86"/>
+      <c r="B18" s="62" t="s">
+        <v>112</v>
+      </c>
+      <c r="C18" s="69" t="s">
+        <v>113</v>
+      </c>
+      <c r="D18" s="87"/>
+      <c r="E18" s="87"/>
+      <c r="F18" s="87"/>
+      <c r="G18" s="87"/>
+      <c r="H18" s="69"/>
     </row>
     <row r="19" spans="1:15" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A19" s="88"/>
-      <c r="B19" s="64"/>
-      <c r="C19" s="71"/>
-      <c r="D19" s="89"/>
-      <c r="E19" s="89"/>
-      <c r="F19" s="89"/>
-      <c r="G19" s="89"/>
-      <c r="H19" s="71"/>
+      <c r="A19" s="86"/>
+      <c r="B19" s="62"/>
+      <c r="C19" s="69"/>
+      <c r="D19" s="87"/>
+      <c r="E19" s="87"/>
+      <c r="F19" s="87"/>
+      <c r="G19" s="87"/>
+      <c r="H19" s="69"/>
     </row>
     <row r="20" spans="1:15" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A20" s="88"/>
-      <c r="B20" s="64"/>
-      <c r="C20" s="71"/>
-      <c r="D20" s="89"/>
-      <c r="E20" s="89"/>
-      <c r="F20" s="89"/>
-      <c r="G20" s="89"/>
-      <c r="H20" s="71"/>
+      <c r="A20" s="86"/>
+      <c r="B20" s="62" t="s">
+        <v>55</v>
+      </c>
+      <c r="C20" s="69" t="s">
+        <v>105</v>
+      </c>
+      <c r="D20" s="87"/>
+      <c r="E20" s="87"/>
+      <c r="F20" s="87"/>
+      <c r="G20" s="87"/>
+      <c r="H20" s="69"/>
     </row>
     <row r="21" spans="1:15" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A21" s="88"/>
-      <c r="B21" s="64"/>
-      <c r="C21" s="71"/>
-      <c r="D21" s="89"/>
-      <c r="E21" s="89"/>
-      <c r="F21" s="89"/>
-      <c r="G21" s="89"/>
-      <c r="H21" s="71"/>
+      <c r="A21" s="86"/>
+      <c r="B21" s="62"/>
+      <c r="C21" s="69"/>
+      <c r="D21" s="87"/>
+      <c r="E21" s="87"/>
+      <c r="F21" s="87"/>
+      <c r="G21" s="87"/>
+      <c r="H21" s="69"/>
     </row>
     <row r="22" spans="1:15" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A22" s="88"/>
-      <c r="B22" s="64"/>
-      <c r="C22" s="71"/>
-      <c r="D22" s="89"/>
-      <c r="E22" s="89"/>
-      <c r="F22" s="89"/>
-      <c r="G22" s="89"/>
-      <c r="H22" s="71"/>
+      <c r="A22" s="86"/>
+      <c r="B22" s="62" t="s">
+        <v>111</v>
+      </c>
+      <c r="C22" s="69" t="s">
+        <v>53</v>
+      </c>
+      <c r="D22" s="87"/>
+      <c r="E22" s="87"/>
+      <c r="F22" s="87"/>
+      <c r="G22" s="87"/>
+      <c r="H22" s="69"/>
     </row>
     <row r="23" spans="1:15" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A23" s="88"/>
-      <c r="B23" s="64"/>
-      <c r="C23" s="71"/>
-      <c r="D23" s="89"/>
-      <c r="E23" s="89"/>
-      <c r="F23" s="89"/>
-      <c r="G23" s="89"/>
-      <c r="H23" s="71"/>
-    </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A24" s="90"/>
-      <c r="B24" s="10"/>
-      <c r="C24" s="11"/>
-      <c r="H24" s="11"/>
-    </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A25" s="90"/>
-      <c r="B25" s="10"/>
-      <c r="C25" s="11"/>
-      <c r="H25" s="11"/>
-    </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A26" s="90"/>
-      <c r="B26" s="10"/>
-      <c r="C26" s="11"/>
-      <c r="H26" s="11"/>
-    </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A27" s="90"/>
-      <c r="B27" s="10"/>
-      <c r="C27" s="11"/>
-      <c r="H27" s="11"/>
-    </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A28" s="90"/>
-      <c r="B28" s="10"/>
-      <c r="C28" s="11"/>
-      <c r="H28" s="11"/>
-    </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A29" s="90"/>
-      <c r="B29" s="10"/>
-      <c r="C29" s="11"/>
-      <c r="H29" s="11"/>
-    </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A30" s="90"/>
+      <c r="A23" s="86"/>
+      <c r="B23" s="62"/>
+      <c r="C23" s="69"/>
+      <c r="D23" s="87"/>
+      <c r="E23" s="87"/>
+      <c r="F23" s="87"/>
+      <c r="G23" s="87"/>
+      <c r="H23" s="69"/>
+      <c r="O23" s="8"/>
+    </row>
+    <row r="24" spans="1:15" ht="15.75" x14ac:dyDescent="0.5">
+      <c r="A24" s="86"/>
+      <c r="B24" s="63" t="s">
+        <v>71</v>
+      </c>
+      <c r="C24" s="69" t="s">
+        <v>53</v>
+      </c>
+      <c r="D24" s="87"/>
+      <c r="E24" s="87"/>
+      <c r="F24" s="87"/>
+      <c r="G24" s="87"/>
+      <c r="H24" s="69"/>
+    </row>
+    <row r="25" spans="1:15" ht="15.75" x14ac:dyDescent="0.5">
+      <c r="A25" s="86"/>
+      <c r="B25" s="63"/>
+      <c r="C25" s="69"/>
+      <c r="D25" s="87"/>
+      <c r="E25" s="87"/>
+      <c r="F25" s="87"/>
+      <c r="G25" s="87"/>
+      <c r="H25" s="69"/>
+    </row>
+    <row r="26" spans="1:15" ht="15.75" x14ac:dyDescent="0.5">
+      <c r="A26" s="86"/>
+      <c r="B26" s="63"/>
+      <c r="C26" s="69"/>
+      <c r="D26" s="87"/>
+      <c r="E26" s="87"/>
+      <c r="F26" s="87"/>
+      <c r="G26" s="87"/>
+      <c r="H26" s="69"/>
+    </row>
+    <row r="27" spans="1:15" ht="15.75" x14ac:dyDescent="0.5">
+      <c r="A27" s="86"/>
+      <c r="B27" s="63"/>
+      <c r="C27" s="69"/>
+      <c r="D27" s="87"/>
+      <c r="E27" s="87"/>
+      <c r="F27" s="87"/>
+      <c r="G27" s="87"/>
+      <c r="H27" s="69"/>
+    </row>
+    <row r="28" spans="1:15" ht="15.75" x14ac:dyDescent="0.5">
+      <c r="A28" s="86"/>
+      <c r="B28" s="63"/>
+      <c r="C28" s="69"/>
+      <c r="D28" s="87"/>
+      <c r="E28" s="87"/>
+      <c r="F28" s="87"/>
+      <c r="G28" s="87"/>
+      <c r="H28" s="69"/>
+    </row>
+    <row r="29" spans="1:15" ht="15.75" x14ac:dyDescent="0.5">
+      <c r="A29" s="86"/>
+      <c r="B29" s="63"/>
+      <c r="C29" s="69"/>
+      <c r="D29" s="87"/>
+      <c r="E29" s="87"/>
+      <c r="F29" s="87"/>
+      <c r="G29" s="87"/>
+      <c r="H29" s="69"/>
+    </row>
+    <row r="30" spans="1:15" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A30" s="89"/>
       <c r="B30" s="10"/>
       <c r="C30" s="11"/>
       <c r="H30" s="11"/>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A31" s="90"/>
+    <row r="31" spans="1:15" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A31" s="89"/>
       <c r="B31" s="10"/>
       <c r="C31" s="11"/>
       <c r="H31" s="11"/>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A32" s="90"/>
+    <row r="32" spans="1:15" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A32" s="89"/>
       <c r="B32" s="10"/>
       <c r="C32" s="11"/>
       <c r="H32" s="11"/>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A33" s="90"/>
+    <row r="33" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A33" s="89"/>
       <c r="B33" s="10"/>
       <c r="C33" s="11"/>
       <c r="H33" s="11"/>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A34" s="90"/>
+    <row r="34" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A34" s="89"/>
       <c r="B34" s="10"/>
       <c r="C34" s="11"/>
       <c r="H34" s="11"/>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A35" s="90"/>
+    <row r="35" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A35" s="89"/>
       <c r="B35" s="10"/>
       <c r="C35" s="11"/>
       <c r="H35" s="11"/>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A36" s="90"/>
+    <row r="36" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A36" s="89"/>
       <c r="B36" s="10"/>
       <c r="C36" s="11"/>
       <c r="H36" s="11"/>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A37" s="90"/>
+    <row r="37" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A37" s="89"/>
       <c r="B37" s="10"/>
       <c r="C37" s="11"/>
       <c r="H37" s="11"/>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A38" s="90"/>
+    <row r="38" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A38" s="89"/>
       <c r="B38" s="10"/>
       <c r="C38" s="11"/>
       <c r="H38" s="11"/>
     </row>
-    <row r="39" spans="1:8" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A39" s="91"/>
-      <c r="B39" s="92"/>
-      <c r="C39" s="93"/>
-      <c r="D39" s="94"/>
-      <c r="E39" s="94"/>
-      <c r="F39" s="94"/>
-      <c r="G39" s="94"/>
-      <c r="H39" s="93"/>
-    </row>
+    <row r="39" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A39" s="89"/>
+      <c r="B39" s="10"/>
+      <c r="C39" s="11"/>
+      <c r="H39" s="11"/>
+    </row>
+    <row r="40" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A40" s="89"/>
+      <c r="B40" s="10"/>
+      <c r="C40" s="11"/>
+      <c r="H40" s="11"/>
+    </row>
+    <row r="41" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A41" s="89"/>
+      <c r="B41" s="10"/>
+      <c r="C41" s="11"/>
+      <c r="H41" s="11"/>
+    </row>
+    <row r="42" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A42" s="89"/>
+      <c r="B42" s="10"/>
+      <c r="C42" s="11"/>
+      <c r="H42" s="11"/>
+    </row>
+    <row r="43" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A43" s="89"/>
+      <c r="B43" s="10"/>
+      <c r="C43" s="11"/>
+      <c r="H43" s="11"/>
+    </row>
+    <row r="44" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A44" s="89"/>
+      <c r="B44" s="10"/>
+      <c r="C44" s="11"/>
+      <c r="H44" s="11"/>
+    </row>
+    <row r="45" spans="1:8" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A45" s="90"/>
+      <c r="B45" s="91"/>
+      <c r="C45" s="92"/>
+      <c r="D45" s="93"/>
+      <c r="E45" s="93"/>
+      <c r="F45" s="93"/>
+      <c r="G45" s="93"/>
+      <c r="H45" s="92"/>
+    </row>
+    <row r="46" spans="1:8" ht="14.25" x14ac:dyDescent="0.45"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="C1:D1"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="42" orientation="portrait" r:id="rId1"/>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:D17"/>
-  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr defaultColWidth="11.3984375" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="3.73046875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="36.73046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.73046875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.73046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.46484375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.86328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="21" x14ac:dyDescent="0.65">
-      <c r="A1" s="103" t="s">
+      <c r="A1" s="110" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="116"/>
+      <c r="C1" s="116"/>
+      <c r="D1" s="117"/>
+    </row>
+    <row r="2" spans="1:4" ht="81.599999999999994" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A2" s="118" t="s">
+        <v>56</v>
+      </c>
+      <c r="B2" s="106"/>
+      <c r="C2" s="106"/>
+      <c r="D2" s="119"/>
+    </row>
+    <row r="3" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
+      <c r="A3" s="59" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" s="60" t="s">
+        <v>57</v>
+      </c>
+      <c r="C3" s="60" t="s">
+        <v>58</v>
+      </c>
+      <c r="D3" s="60" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
+      <c r="A4" s="61">
+        <v>1</v>
+      </c>
+      <c r="B4" s="94" t="s">
+        <v>59</v>
+      </c>
+      <c r="C4" s="65">
+        <v>0</v>
+      </c>
+      <c r="D4" s="65">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
+      <c r="A5" s="61">
+        <v>2</v>
+      </c>
+      <c r="B5" s="62" t="s">
+        <v>73</v>
+      </c>
+      <c r="C5" s="65">
+        <v>50</v>
+      </c>
+      <c r="D5" s="65"/>
+    </row>
+    <row r="6" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
+      <c r="A6" s="61">
+        <v>3</v>
+      </c>
+      <c r="B6" s="62" t="s">
+        <v>75</v>
+      </c>
+      <c r="C6" s="65">
+        <v>40</v>
+      </c>
+      <c r="D6" s="65"/>
+    </row>
+    <row r="7" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
+      <c r="A7" s="61">
+        <v>4</v>
+      </c>
+      <c r="B7" s="62" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7" s="65">
         <v>20</v>
       </c>
-      <c r="B1" s="109"/>
-      <c r="C1" s="109"/>
-      <c r="D1" s="110"/>
-    </row>
-    <row r="2" spans="1:4" ht="81.599999999999994" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="111" t="s">
-        <v>44</v>
-      </c>
-      <c r="B2" s="112"/>
-      <c r="C2" s="112"/>
-      <c r="D2" s="113"/>
-    </row>
-    <row r="3" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A3" s="60" t="s">
-        <v>25</v>
-      </c>
-      <c r="B3" s="61" t="s">
-        <v>29</v>
-      </c>
-      <c r="C3" s="61" t="s">
-        <v>31</v>
-      </c>
-      <c r="D3" s="61" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A4" s="62">
-        <v>1</v>
-      </c>
-      <c r="B4" s="95" t="s">
-        <v>47</v>
-      </c>
-      <c r="C4" s="66">
-        <v>0</v>
-      </c>
-      <c r="D4" s="66">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A5" s="62">
-        <v>2</v>
-      </c>
-      <c r="B5" s="63" t="s">
-        <v>81</v>
-      </c>
-      <c r="C5" s="66">
-        <v>50</v>
-      </c>
-      <c r="D5" s="66"/>
-    </row>
-    <row r="6" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A6" s="62">
-        <v>3</v>
-      </c>
-      <c r="B6" s="63" t="s">
-        <v>83</v>
-      </c>
-      <c r="C6" s="66">
-        <v>40</v>
-      </c>
-      <c r="D6" s="66"/>
-    </row>
-    <row r="7" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A7" s="62">
-        <v>4</v>
-      </c>
-      <c r="B7" s="63" t="s">
-        <v>80</v>
-      </c>
-      <c r="C7" s="66">
-        <v>20</v>
-      </c>
-      <c r="D7" s="66"/>
+      <c r="D7" s="65"/>
     </row>
     <row r="8" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A8" s="62">
+      <c r="A8" s="61">
         <v>5</v>
       </c>
-      <c r="B8" s="63" t="s">
-        <v>82</v>
-      </c>
-      <c r="C8" s="66">
+      <c r="B8" s="62" t="s">
+        <v>74</v>
+      </c>
+      <c r="C8" s="65">
         <v>10</v>
       </c>
-      <c r="D8" s="66"/>
+      <c r="D8" s="65"/>
     </row>
     <row r="9" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A9" s="62"/>
-      <c r="B9" s="63"/>
-      <c r="C9" s="66"/>
-      <c r="D9" s="66"/>
+      <c r="A9" s="61"/>
+      <c r="B9" s="62"/>
+      <c r="C9" s="65"/>
+      <c r="D9" s="65"/>
     </row>
     <row r="10" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A10" s="62"/>
-      <c r="B10" s="63"/>
-      <c r="C10" s="66"/>
-      <c r="D10" s="66"/>
+      <c r="A10" s="61"/>
+      <c r="B10" s="62"/>
+      <c r="C10" s="65"/>
+      <c r="D10" s="65"/>
     </row>
     <row r="11" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A11" s="62"/>
-      <c r="B11" s="63"/>
-      <c r="C11" s="66"/>
-      <c r="D11" s="66"/>
+      <c r="A11" s="61"/>
+      <c r="B11" s="62"/>
+      <c r="C11" s="65"/>
+      <c r="D11" s="65"/>
     </row>
     <row r="12" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A12" s="62"/>
-      <c r="B12" s="63"/>
-      <c r="C12" s="66"/>
-      <c r="D12" s="66"/>
+      <c r="A12" s="61"/>
+      <c r="B12" s="62"/>
+      <c r="C12" s="65"/>
+      <c r="D12" s="65"/>
     </row>
     <row r="13" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A13" s="62"/>
-      <c r="B13" s="63"/>
-      <c r="C13" s="66"/>
-      <c r="D13" s="66"/>
+      <c r="A13" s="61"/>
+      <c r="B13" s="62"/>
+      <c r="C13" s="65"/>
+      <c r="D13" s="65"/>
     </row>
     <row r="14" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A14" s="62"/>
-      <c r="B14" s="63"/>
-      <c r="C14" s="66"/>
-      <c r="D14" s="66"/>
+      <c r="A14" s="61"/>
+      <c r="B14" s="62"/>
+      <c r="C14" s="65"/>
+      <c r="D14" s="65"/>
     </row>
     <row r="15" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A15" s="62"/>
-      <c r="B15" s="63"/>
-      <c r="C15" s="66"/>
-      <c r="D15" s="66"/>
+      <c r="A15" s="61"/>
+      <c r="B15" s="62"/>
+      <c r="C15" s="65"/>
+      <c r="D15" s="65"/>
     </row>
     <row r="16" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A16" s="62"/>
-      <c r="B16" s="63"/>
-      <c r="C16" s="66"/>
-      <c r="D16" s="66"/>
+      <c r="A16" s="61"/>
+      <c r="B16" s="62"/>
+      <c r="C16" s="65"/>
+      <c r="D16" s="65"/>
     </row>
     <row r="17" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="A17" s="65"/>
-      <c r="B17" s="61" t="s">
-        <v>30</v>
-      </c>
-      <c r="C17" s="67">
+      <c r="A17" s="64"/>
+      <c r="B17" s="60" t="s">
+        <v>60</v>
+      </c>
+      <c r="C17" s="66">
         <f>SUM(C4:C16)</f>
         <v>120</v>
       </c>
-      <c r="D17" s="67">
+      <c r="D17" s="66">
         <f>SUM(D4:D16)</f>
         <v>0</v>
       </c>
     </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="B18" s="122" t="s">
+        <v>116</v>
+      </c>
+      <c r="C18" s="122"/>
+      <c r="D18" s="122"/>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C1:D1"/>
     <mergeCell ref="A2:D2"/>
+    <mergeCell ref="B18:D18"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
@@ -4128,72 +4682,72 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:H8"/>
-  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="11.3984375" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="11.3984375" style="1"/>
     <col min="2" max="2" width="41.265625" customWidth="1"/>
     <col min="3" max="5" width="21.265625" customWidth="1"/>
     <col min="6" max="6" width="49.3984375" customWidth="1"/>
     <col min="7" max="7" width="31.3984375" customWidth="1"/>
-    <col min="8" max="8" width="14.265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="28.59765625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="21" x14ac:dyDescent="0.65">
-      <c r="A1" s="103" t="s">
-        <v>23</v>
-      </c>
-      <c r="B1" s="109"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
+      <c r="A1" s="110" t="s">
+        <v>61</v>
+      </c>
+      <c r="B1" s="116"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
     </row>
     <row r="2" spans="1:8" ht="57" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="118" t="s">
-        <v>42</v>
-      </c>
-      <c r="B2" s="119"/>
-      <c r="C2" s="119"/>
-      <c r="D2" s="119"/>
-      <c r="E2" s="119"/>
-      <c r="F2" s="119"/>
-      <c r="G2" s="119"/>
-      <c r="H2" s="119"/>
+      <c r="A2" s="120" t="s">
+        <v>62</v>
+      </c>
+      <c r="B2" s="121"/>
+      <c r="C2" s="121"/>
+      <c r="D2" s="121"/>
+      <c r="E2" s="121"/>
+      <c r="F2" s="121"/>
+      <c r="G2" s="121"/>
+      <c r="H2" s="121"/>
     </row>
     <row r="3" spans="1:8" s="2" customFormat="1" ht="47.25" x14ac:dyDescent="0.45">
       <c r="A3" s="31" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B3" s="32" t="s">
-        <v>0</v>
+        <v>63</v>
       </c>
       <c r="C3" s="33" t="s">
-        <v>36</v>
+        <v>64</v>
       </c>
       <c r="D3" s="33" t="s">
-        <v>37</v>
+        <v>65</v>
       </c>
       <c r="E3" s="33" t="s">
-        <v>34</v>
+        <v>66</v>
       </c>
       <c r="F3" s="32" t="s">
-        <v>35</v>
+        <v>67</v>
       </c>
       <c r="G3" s="32" t="s">
-        <v>27</v>
+        <v>46</v>
       </c>
       <c r="H3" s="33" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="25.15" customHeight="1" x14ac:dyDescent="0.45">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="34">
         <v>1</v>
       </c>
       <c r="B4" s="35" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="C4" s="36">
         <v>0.05</v>
@@ -4205,22 +4759,24 @@
         <v>1</v>
       </c>
       <c r="F4" s="37" t="s">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="G4" s="37" t="s">
-        <v>86</v>
-      </c>
-      <c r="H4" s="38"/>
+        <v>53</v>
+      </c>
+      <c r="H4" s="124" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="5" spans="1:8" ht="31.5" x14ac:dyDescent="0.45">
       <c r="A5" s="34">
         <v>2</v>
       </c>
       <c r="B5" s="35" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C5" s="36" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D5" s="36">
         <v>0.6</v>
@@ -4228,20 +4784,22 @@
       <c r="E5" s="36">
         <v>0.8</v>
       </c>
-      <c r="F5" s="37" t="s">
-        <v>90</v>
+      <c r="F5" s="123" t="s">
+        <v>119</v>
       </c>
       <c r="G5" s="37" t="s">
-        <v>40</v>
-      </c>
-      <c r="H5" s="38"/>
+        <v>117</v>
+      </c>
+      <c r="H5" s="124" t="s">
+        <v>123</v>
+      </c>
     </row>
     <row r="6" spans="1:8" ht="25.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="34">
         <v>3</v>
       </c>
       <c r="B6" s="35" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="C6" s="36">
         <v>0.1</v>
@@ -4253,43 +4811,47 @@
         <v>0.15</v>
       </c>
       <c r="F6" s="37" t="s">
-        <v>95</v>
+        <v>81</v>
       </c>
       <c r="G6" s="37" t="s">
-        <v>89</v>
-      </c>
-      <c r="H6" s="38"/>
-    </row>
-    <row r="7" spans="1:8" ht="25.15" customHeight="1" x14ac:dyDescent="0.45">
+        <v>114</v>
+      </c>
+      <c r="H6" s="124">
+        <v>46214</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="35.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="34">
         <v>4</v>
       </c>
       <c r="B7" s="35" t="s">
-        <v>93</v>
+        <v>79</v>
       </c>
       <c r="C7" s="36">
         <v>0.01</v>
       </c>
       <c r="D7" s="36" t="s">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="E7" s="36">
         <v>0.5</v>
       </c>
-      <c r="F7" s="37" t="s">
-        <v>92</v>
+      <c r="F7" s="123" t="s">
+        <v>120</v>
       </c>
       <c r="G7" s="37" t="s">
-        <v>88</v>
-      </c>
-      <c r="H7" s="38"/>
-    </row>
-    <row r="8" spans="1:8" ht="25.15" customHeight="1" x14ac:dyDescent="0.45">
+        <v>107</v>
+      </c>
+      <c r="H7" s="124">
+        <v>46173</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="39" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="34">
         <v>5</v>
       </c>
       <c r="B8" s="35" t="s">
-        <v>96</v>
+        <v>82</v>
       </c>
       <c r="C8" s="36">
         <v>0.3</v>
@@ -4300,20 +4862,22 @@
       <c r="E8" s="36">
         <v>1</v>
       </c>
-      <c r="F8" s="37" t="s">
-        <v>97</v>
+      <c r="F8" s="123" t="s">
+        <v>121</v>
       </c>
       <c r="G8" s="37" t="s">
-        <v>87</v>
-      </c>
-      <c r="H8" s="38"/>
+        <v>118</v>
+      </c>
+      <c r="H8" s="124">
+        <v>46174</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:H2"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="51" orientation="portrait" r:id="rId1"/>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>